<commit_message>
Adding CSV and Json DDT
</commit_message>
<xml_diff>
--- a/playwright-framework/src/data/ddt/generated/ddt-data.xlsx
+++ b/playwright-framework/src/data/ddt/generated/ddt-data.xlsx
@@ -47,7 +47,7 @@
     <t>testuser1@test.com</t>
   </si>
   <si>
-    <t>0533213903</t>
+    <t>0596639158</t>
   </si>
   <si>
     <t>City1</t>
@@ -65,7 +65,7 @@
     <t>testuser2@test.com</t>
   </si>
   <si>
-    <t>0519713610</t>
+    <t>0580407018</t>
   </si>
   <si>
     <t>City2</t>
@@ -83,7 +83,7 @@
     <t>testuser3@test.com</t>
   </si>
   <si>
-    <t>0521165072</t>
+    <t>0548123541</t>
   </si>
   <si>
     <t>City3</t>
@@ -101,7 +101,7 @@
     <t>testuser4@test.com</t>
   </si>
   <si>
-    <t>0579061965</t>
+    <t>0536052129</t>
   </si>
   <si>
     <t>City4</t>
@@ -119,7 +119,7 @@
     <t>testuser5@test.com</t>
   </si>
   <si>
-    <t>0594744006</t>
+    <t>0590441624</t>
   </si>
   <si>
     <t>City5</t>
@@ -137,7 +137,7 @@
     <t>testuser6@test.com</t>
   </si>
   <si>
-    <t>0569195206</t>
+    <t>0553704354</t>
   </si>
   <si>
     <t>City6</t>
@@ -152,7 +152,7 @@
     <t>testuser7@test.com</t>
   </si>
   <si>
-    <t>0594083383</t>
+    <t>0510603651</t>
   </si>
   <si>
     <t>City7</t>
@@ -167,7 +167,7 @@
     <t>testuser8@test.com</t>
   </si>
   <si>
-    <t>0592361186</t>
+    <t>0577822050</t>
   </si>
   <si>
     <t>City8</t>
@@ -182,7 +182,7 @@
     <t>testuser9@test.com</t>
   </si>
   <si>
-    <t>0566995958</t>
+    <t>0516443431</t>
   </si>
   <si>
     <t>City9</t>
@@ -197,7 +197,7 @@
     <t>testuser10@test.com</t>
   </si>
   <si>
-    <t>0522066062</t>
+    <t>0535451764</t>
   </si>
   <si>
     <t>City10</t>
@@ -212,7 +212,7 @@
     <t>testuser11@test.com</t>
   </si>
   <si>
-    <t>0599990602</t>
+    <t>0585846924</t>
   </si>
   <si>
     <t>City11</t>
@@ -227,7 +227,7 @@
     <t>testuser12@test.com</t>
   </si>
   <si>
-    <t>0562294828</t>
+    <t>0575467399</t>
   </si>
   <si>
     <t>City12</t>
@@ -242,7 +242,7 @@
     <t>testuser13@test.com</t>
   </si>
   <si>
-    <t>0587498038</t>
+    <t>0532974086</t>
   </si>
   <si>
     <t>City13</t>
@@ -257,7 +257,7 @@
     <t>testuser14@test.com</t>
   </si>
   <si>
-    <t>0566001493</t>
+    <t>0533535775</t>
   </si>
   <si>
     <t>City14</t>
@@ -272,7 +272,7 @@
     <t>testuser15@test.com</t>
   </si>
   <si>
-    <t>0567151357</t>
+    <t>0570158499</t>
   </si>
   <si>
     <t>City15</t>
@@ -287,7 +287,7 @@
     <t>testuser16@test.com</t>
   </si>
   <si>
-    <t>0579338357</t>
+    <t>0590998526</t>
   </si>
   <si>
     <t>City16</t>
@@ -302,7 +302,7 @@
     <t>testuser17@test.com</t>
   </si>
   <si>
-    <t>0571657963</t>
+    <t>0525262356</t>
   </si>
   <si>
     <t>City17</t>
@@ -317,7 +317,7 @@
     <t>testuser18@test.com</t>
   </si>
   <si>
-    <t>0561469773</t>
+    <t>0516165906</t>
   </si>
   <si>
     <t>City18</t>
@@ -332,7 +332,7 @@
     <t>testuser19@test.com</t>
   </si>
   <si>
-    <t>0542379092</t>
+    <t>0585977150</t>
   </si>
   <si>
     <t>City19</t>
@@ -347,7 +347,7 @@
     <t>testuser20@test.com</t>
   </si>
   <si>
-    <t>0590688820</t>
+    <t>0568122001</t>
   </si>
   <si>
     <t>City20</t>
@@ -362,7 +362,7 @@
     <t>testuser21@test.com</t>
   </si>
   <si>
-    <t>0554969273</t>
+    <t>0533727474</t>
   </si>
   <si>
     <t>City21</t>
@@ -377,7 +377,7 @@
     <t>testuser22@test.com</t>
   </si>
   <si>
-    <t>0534880565</t>
+    <t>0516153368</t>
   </si>
   <si>
     <t>City22</t>
@@ -392,7 +392,7 @@
     <t>testuser23@test.com</t>
   </si>
   <si>
-    <t>0587191120</t>
+    <t>0562048836</t>
   </si>
   <si>
     <t>City23</t>
@@ -407,7 +407,7 @@
     <t>testuser24@test.com</t>
   </si>
   <si>
-    <t>0513776183</t>
+    <t>0514664706</t>
   </si>
   <si>
     <t>City24</t>
@@ -422,7 +422,7 @@
     <t>testuser25@test.com</t>
   </si>
   <si>
-    <t>0596442901</t>
+    <t>0529888801</t>
   </si>
   <si>
     <t>City25</t>
@@ -437,7 +437,7 @@
     <t>testuser26@test.com</t>
   </si>
   <si>
-    <t>0543397858</t>
+    <t>0533564177</t>
   </si>
   <si>
     <t>City26</t>
@@ -452,7 +452,7 @@
     <t>testuser27@test.com</t>
   </si>
   <si>
-    <t>0550462357</t>
+    <t>0538562968</t>
   </si>
   <si>
     <t>City27</t>
@@ -467,7 +467,7 @@
     <t>testuser28@test.com</t>
   </si>
   <si>
-    <t>0531054232</t>
+    <t>0531830745</t>
   </si>
   <si>
     <t>City28</t>
@@ -482,7 +482,7 @@
     <t>testuser29@test.com</t>
   </si>
   <si>
-    <t>0589510984</t>
+    <t>0568780382</t>
   </si>
   <si>
     <t>City29</t>
@@ -497,7 +497,7 @@
     <t>testuser30@test.com</t>
   </si>
   <si>
-    <t>0566965063</t>
+    <t>0533764210</t>
   </si>
   <si>
     <t>City30</t>
@@ -512,7 +512,7 @@
     <t>testuser31@test.com</t>
   </si>
   <si>
-    <t>0576701996</t>
+    <t>0598462940</t>
   </si>
   <si>
     <t>City31</t>
@@ -527,7 +527,7 @@
     <t>testuser32@test.com</t>
   </si>
   <si>
-    <t>0599165132</t>
+    <t>0532546004</t>
   </si>
   <si>
     <t>City32</t>
@@ -542,7 +542,7 @@
     <t>testuser33@test.com</t>
   </si>
   <si>
-    <t>0566177130</t>
+    <t>0589178791</t>
   </si>
   <si>
     <t>City33</t>
@@ -557,7 +557,7 @@
     <t>testuser34@test.com</t>
   </si>
   <si>
-    <t>0543761976</t>
+    <t>0514464983</t>
   </si>
   <si>
     <t>City34</t>
@@ -572,7 +572,7 @@
     <t>testuser35@test.com</t>
   </si>
   <si>
-    <t>0572857684</t>
+    <t>0551090969</t>
   </si>
   <si>
     <t>City35</t>
@@ -587,7 +587,7 @@
     <t>testuser36@test.com</t>
   </si>
   <si>
-    <t>0547078327</t>
+    <t>0592903771</t>
   </si>
   <si>
     <t>City36</t>
@@ -602,7 +602,7 @@
     <t>testuser37@test.com</t>
   </si>
   <si>
-    <t>0531538949</t>
+    <t>0525130556</t>
   </si>
   <si>
     <t>City37</t>
@@ -617,7 +617,7 @@
     <t>testuser38@test.com</t>
   </si>
   <si>
-    <t>0583624404</t>
+    <t>0587144516</t>
   </si>
   <si>
     <t>City38</t>
@@ -632,7 +632,7 @@
     <t>testuser39@test.com</t>
   </si>
   <si>
-    <t>0572246020</t>
+    <t>0510251417</t>
   </si>
   <si>
     <t>City39</t>
@@ -647,7 +647,7 @@
     <t>testuser40@test.com</t>
   </si>
   <si>
-    <t>0542094172</t>
+    <t>0582564354</t>
   </si>
   <si>
     <t>City40</t>
@@ -662,7 +662,7 @@
     <t>testuser41@test.com</t>
   </si>
   <si>
-    <t>0570729030</t>
+    <t>0560614167</t>
   </si>
   <si>
     <t>City41</t>
@@ -677,7 +677,7 @@
     <t>testuser42@test.com</t>
   </si>
   <si>
-    <t>0543355102</t>
+    <t>0519964808</t>
   </si>
   <si>
     <t>City42</t>
@@ -692,7 +692,7 @@
     <t>testuser43@test.com</t>
   </si>
   <si>
-    <t>0525102450</t>
+    <t>0546618505</t>
   </si>
   <si>
     <t>City43</t>
@@ -707,7 +707,7 @@
     <t>testuser44@test.com</t>
   </si>
   <si>
-    <t>0517357301</t>
+    <t>0544514801</t>
   </si>
   <si>
     <t>City44</t>
@@ -722,7 +722,7 @@
     <t>testuser45@test.com</t>
   </si>
   <si>
-    <t>0525771646</t>
+    <t>0510190870</t>
   </si>
   <si>
     <t>City45</t>
@@ -737,7 +737,7 @@
     <t>testuser46@test.com</t>
   </si>
   <si>
-    <t>0572782212</t>
+    <t>0536267672</t>
   </si>
   <si>
     <t>City46</t>
@@ -752,7 +752,7 @@
     <t>testuser47@test.com</t>
   </si>
   <si>
-    <t>0564163028</t>
+    <t>0521008561</t>
   </si>
   <si>
     <t>City47</t>
@@ -767,7 +767,7 @@
     <t>testuser48@test.com</t>
   </si>
   <si>
-    <t>0560443038</t>
+    <t>0540676138</t>
   </si>
   <si>
     <t>City48</t>
@@ -782,7 +782,7 @@
     <t>testuser49@test.com</t>
   </si>
   <si>
-    <t>0588559772</t>
+    <t>0528792790</t>
   </si>
   <si>
     <t>City49</t>
@@ -797,7 +797,7 @@
     <t>testuser50@test.com</t>
   </si>
   <si>
-    <t>0523848644</t>
+    <t>0564500861</t>
   </si>
   <si>
     <t>City50</t>
@@ -1562,7 +1562,7 @@
         <v>13</v>
       </c>
       <c r="G2">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="H2" t="b">
         <v>0</v>
@@ -1588,7 +1588,7 @@
         <v>19</v>
       </c>
       <c r="G3">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="H3" t="b">
         <v>1</v>
@@ -1614,7 +1614,7 @@
         <v>25</v>
       </c>
       <c r="G4">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="H4" t="b">
         <v>0</v>
@@ -1640,7 +1640,7 @@
         <v>31</v>
       </c>
       <c r="G5">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="H5" t="b">
         <v>1</v>
@@ -1666,7 +1666,7 @@
         <v>37</v>
       </c>
       <c r="G6">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="H6" t="b">
         <v>0</v>
@@ -1692,7 +1692,7 @@
         <v>13</v>
       </c>
       <c r="G7">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H7" t="b">
         <v>1</v>
@@ -1718,7 +1718,7 @@
         <v>19</v>
       </c>
       <c r="G8">
-        <v>64</v>
+        <v>45</v>
       </c>
       <c r="H8" t="b">
         <v>0</v>
@@ -1744,7 +1744,7 @@
         <v>25</v>
       </c>
       <c r="G9">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="H9" t="b">
         <v>1</v>
@@ -1770,7 +1770,7 @@
         <v>31</v>
       </c>
       <c r="G10">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="H10" t="b">
         <v>0</v>
@@ -1796,7 +1796,7 @@
         <v>37</v>
       </c>
       <c r="G11">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="H11" t="b">
         <v>1</v>
@@ -1822,7 +1822,7 @@
         <v>13</v>
       </c>
       <c r="G12">
-        <v>26</v>
+        <v>43</v>
       </c>
       <c r="H12" t="b">
         <v>0</v>
@@ -1848,7 +1848,7 @@
         <v>19</v>
       </c>
       <c r="G13">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="H13" t="b">
         <v>1</v>
@@ -1874,7 +1874,7 @@
         <v>25</v>
       </c>
       <c r="G14">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="H14" t="b">
         <v>0</v>
@@ -1900,7 +1900,7 @@
         <v>31</v>
       </c>
       <c r="G15">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="H15" t="b">
         <v>1</v>
@@ -1926,7 +1926,7 @@
         <v>37</v>
       </c>
       <c r="G16">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="H16" t="b">
         <v>0</v>
@@ -1952,7 +1952,7 @@
         <v>13</v>
       </c>
       <c r="G17">
-        <v>57</v>
+        <v>19</v>
       </c>
       <c r="H17" t="b">
         <v>1</v>
@@ -1978,7 +1978,7 @@
         <v>19</v>
       </c>
       <c r="G18">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="H18" t="b">
         <v>0</v>
@@ -2004,7 +2004,7 @@
         <v>25</v>
       </c>
       <c r="G19">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="H19" t="b">
         <v>1</v>
@@ -2030,7 +2030,7 @@
         <v>31</v>
       </c>
       <c r="G20">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="H20" t="b">
         <v>0</v>
@@ -2056,7 +2056,7 @@
         <v>37</v>
       </c>
       <c r="G21">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="H21" t="b">
         <v>1</v>
@@ -2082,7 +2082,7 @@
         <v>13</v>
       </c>
       <c r="G22">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="H22" t="b">
         <v>0</v>
@@ -2108,7 +2108,7 @@
         <v>19</v>
       </c>
       <c r="G23">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="H23" t="b">
         <v>1</v>
@@ -2134,7 +2134,7 @@
         <v>25</v>
       </c>
       <c r="G24">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="H24" t="b">
         <v>0</v>
@@ -2160,7 +2160,7 @@
         <v>31</v>
       </c>
       <c r="G25">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="H25" t="b">
         <v>1</v>
@@ -2186,7 +2186,7 @@
         <v>37</v>
       </c>
       <c r="G26">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="H26" t="b">
         <v>0</v>
@@ -2212,7 +2212,7 @@
         <v>13</v>
       </c>
       <c r="G27">
-        <v>24</v>
+        <v>43</v>
       </c>
       <c r="H27" t="b">
         <v>1</v>
@@ -2238,7 +2238,7 @@
         <v>19</v>
       </c>
       <c r="G28">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="H28" t="b">
         <v>0</v>
@@ -2264,7 +2264,7 @@
         <v>25</v>
       </c>
       <c r="G29">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="H29" t="b">
         <v>1</v>
@@ -2290,7 +2290,7 @@
         <v>31</v>
       </c>
       <c r="G30">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="H30" t="b">
         <v>0</v>
@@ -2316,7 +2316,7 @@
         <v>37</v>
       </c>
       <c r="G31">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="H31" t="b">
         <v>1</v>
@@ -2342,7 +2342,7 @@
         <v>13</v>
       </c>
       <c r="G32">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="H32" t="b">
         <v>0</v>
@@ -2368,7 +2368,7 @@
         <v>19</v>
       </c>
       <c r="G33">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="H33" t="b">
         <v>1</v>
@@ -2394,7 +2394,7 @@
         <v>25</v>
       </c>
       <c r="G34">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="H34" t="b">
         <v>0</v>
@@ -2420,7 +2420,7 @@
         <v>31</v>
       </c>
       <c r="G35">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="H35" t="b">
         <v>1</v>
@@ -2446,7 +2446,7 @@
         <v>37</v>
       </c>
       <c r="G36">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="H36" t="b">
         <v>0</v>
@@ -2472,7 +2472,7 @@
         <v>13</v>
       </c>
       <c r="G37">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="H37" t="b">
         <v>1</v>
@@ -2498,7 +2498,7 @@
         <v>19</v>
       </c>
       <c r="G38">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="H38" t="b">
         <v>0</v>
@@ -2524,7 +2524,7 @@
         <v>25</v>
       </c>
       <c r="G39">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="H39" t="b">
         <v>1</v>
@@ -2550,7 +2550,7 @@
         <v>31</v>
       </c>
       <c r="G40">
-        <v>35</v>
+        <v>58</v>
       </c>
       <c r="H40" t="b">
         <v>0</v>
@@ -2602,7 +2602,7 @@
         <v>13</v>
       </c>
       <c r="G42">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="H42" t="b">
         <v>0</v>
@@ -2628,7 +2628,7 @@
         <v>19</v>
       </c>
       <c r="G43">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="H43" t="b">
         <v>1</v>
@@ -2654,7 +2654,7 @@
         <v>25</v>
       </c>
       <c r="G44">
-        <v>21</v>
+        <v>56</v>
       </c>
       <c r="H44" t="b">
         <v>0</v>
@@ -2680,7 +2680,7 @@
         <v>31</v>
       </c>
       <c r="G45">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="H45" t="b">
         <v>1</v>
@@ -2706,7 +2706,7 @@
         <v>37</v>
       </c>
       <c r="G46">
-        <v>54</v>
+        <v>27</v>
       </c>
       <c r="H46" t="b">
         <v>0</v>
@@ -2732,7 +2732,7 @@
         <v>13</v>
       </c>
       <c r="G47">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H47" t="b">
         <v>1</v>
@@ -2758,7 +2758,7 @@
         <v>19</v>
       </c>
       <c r="G48">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="H48" t="b">
         <v>0</v>
@@ -2784,7 +2784,7 @@
         <v>25</v>
       </c>
       <c r="G49">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="H49" t="b">
         <v>1</v>
@@ -2810,7 +2810,7 @@
         <v>31</v>
       </c>
       <c r="G50">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="H50" t="b">
         <v>0</v>
@@ -2836,7 +2836,7 @@
         <v>37</v>
       </c>
       <c r="G51">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="H51" t="b">
         <v>1</v>
@@ -2881,7 +2881,7 @@
         <v>269</v>
       </c>
       <c r="C2">
-        <v>404</v>
+        <v>122</v>
       </c>
       <c r="D2" t="s">
         <v>270</v>
@@ -2898,7 +2898,7 @@
         <v>272</v>
       </c>
       <c r="C3">
-        <v>307</v>
+        <v>282</v>
       </c>
       <c r="D3" t="s">
         <v>273</v>
@@ -2915,7 +2915,7 @@
         <v>275</v>
       </c>
       <c r="C4">
-        <v>779</v>
+        <v>655</v>
       </c>
       <c r="D4" t="s">
         <v>276</v>
@@ -2932,7 +2932,7 @@
         <v>278</v>
       </c>
       <c r="C5">
-        <v>448</v>
+        <v>569</v>
       </c>
       <c r="D5" t="s">
         <v>279</v>
@@ -2949,7 +2949,7 @@
         <v>281</v>
       </c>
       <c r="C6">
-        <v>251</v>
+        <v>110</v>
       </c>
       <c r="D6" t="s">
         <v>270</v>
@@ -2966,7 +2966,7 @@
         <v>283</v>
       </c>
       <c r="C7">
-        <v>673</v>
+        <v>825</v>
       </c>
       <c r="D7" t="s">
         <v>273</v>
@@ -2983,7 +2983,7 @@
         <v>285</v>
       </c>
       <c r="C8">
-        <v>517</v>
+        <v>426</v>
       </c>
       <c r="D8" t="s">
         <v>276</v>
@@ -3000,7 +3000,7 @@
         <v>287</v>
       </c>
       <c r="C9">
-        <v>685</v>
+        <v>972</v>
       </c>
       <c r="D9" t="s">
         <v>279</v>
@@ -3017,7 +3017,7 @@
         <v>289</v>
       </c>
       <c r="C10">
-        <v>469</v>
+        <v>768</v>
       </c>
       <c r="D10" t="s">
         <v>270</v>
@@ -3034,7 +3034,7 @@
         <v>291</v>
       </c>
       <c r="C11">
-        <v>468</v>
+        <v>141</v>
       </c>
       <c r="D11" t="s">
         <v>273</v>
@@ -3051,7 +3051,7 @@
         <v>293</v>
       </c>
       <c r="C12">
-        <v>807</v>
+        <v>148</v>
       </c>
       <c r="D12" t="s">
         <v>276</v>
@@ -3068,7 +3068,7 @@
         <v>295</v>
       </c>
       <c r="C13">
-        <v>699</v>
+        <v>419</v>
       </c>
       <c r="D13" t="s">
         <v>279</v>
@@ -3085,7 +3085,7 @@
         <v>297</v>
       </c>
       <c r="C14">
-        <v>668</v>
+        <v>899</v>
       </c>
       <c r="D14" t="s">
         <v>270</v>
@@ -3102,7 +3102,7 @@
         <v>299</v>
       </c>
       <c r="C15">
-        <v>208</v>
+        <v>10</v>
       </c>
       <c r="D15" t="s">
         <v>273</v>
@@ -3119,7 +3119,7 @@
         <v>301</v>
       </c>
       <c r="C16">
-        <v>312</v>
+        <v>847</v>
       </c>
       <c r="D16" t="s">
         <v>276</v>
@@ -3136,7 +3136,7 @@
         <v>303</v>
       </c>
       <c r="C17">
-        <v>824</v>
+        <v>563</v>
       </c>
       <c r="D17" t="s">
         <v>279</v>
@@ -3153,7 +3153,7 @@
         <v>305</v>
       </c>
       <c r="C18">
-        <v>96</v>
+        <v>315</v>
       </c>
       <c r="D18" t="s">
         <v>270</v>
@@ -3170,7 +3170,7 @@
         <v>307</v>
       </c>
       <c r="C19">
-        <v>899</v>
+        <v>121</v>
       </c>
       <c r="D19" t="s">
         <v>273</v>
@@ -3187,7 +3187,7 @@
         <v>309</v>
       </c>
       <c r="C20">
-        <v>113</v>
+        <v>318</v>
       </c>
       <c r="D20" t="s">
         <v>276</v>
@@ -3204,7 +3204,7 @@
         <v>311</v>
       </c>
       <c r="C21">
-        <v>323</v>
+        <v>332</v>
       </c>
       <c r="D21" t="s">
         <v>279</v>
@@ -3221,7 +3221,7 @@
         <v>313</v>
       </c>
       <c r="C22">
-        <v>180</v>
+        <v>948</v>
       </c>
       <c r="D22" t="s">
         <v>270</v>
@@ -3238,7 +3238,7 @@
         <v>315</v>
       </c>
       <c r="C23">
-        <v>927</v>
+        <v>378</v>
       </c>
       <c r="D23" t="s">
         <v>273</v>
@@ -3255,7 +3255,7 @@
         <v>317</v>
       </c>
       <c r="C24">
-        <v>737</v>
+        <v>914</v>
       </c>
       <c r="D24" t="s">
         <v>276</v>
@@ -3272,7 +3272,7 @@
         <v>319</v>
       </c>
       <c r="C25">
-        <v>285</v>
+        <v>432</v>
       </c>
       <c r="D25" t="s">
         <v>279</v>
@@ -3289,7 +3289,7 @@
         <v>321</v>
       </c>
       <c r="C26">
-        <v>670</v>
+        <v>555</v>
       </c>
       <c r="D26" t="s">
         <v>270</v>
@@ -3306,7 +3306,7 @@
         <v>323</v>
       </c>
       <c r="C27">
-        <v>622</v>
+        <v>921</v>
       </c>
       <c r="D27" t="s">
         <v>273</v>
@@ -3323,7 +3323,7 @@
         <v>325</v>
       </c>
       <c r="C28">
-        <v>287</v>
+        <v>794</v>
       </c>
       <c r="D28" t="s">
         <v>276</v>
@@ -3340,7 +3340,7 @@
         <v>327</v>
       </c>
       <c r="C29">
-        <v>154</v>
+        <v>416</v>
       </c>
       <c r="D29" t="s">
         <v>279</v>
@@ -3357,7 +3357,7 @@
         <v>329</v>
       </c>
       <c r="C30">
-        <v>851</v>
+        <v>620</v>
       </c>
       <c r="D30" t="s">
         <v>270</v>
@@ -3374,7 +3374,7 @@
         <v>331</v>
       </c>
       <c r="C31">
-        <v>830</v>
+        <v>929</v>
       </c>
       <c r="D31" t="s">
         <v>273</v>
@@ -3391,7 +3391,7 @@
         <v>333</v>
       </c>
       <c r="C32">
-        <v>153</v>
+        <v>488</v>
       </c>
       <c r="D32" t="s">
         <v>276</v>
@@ -3408,7 +3408,7 @@
         <v>335</v>
       </c>
       <c r="C33">
-        <v>557</v>
+        <v>257</v>
       </c>
       <c r="D33" t="s">
         <v>279</v>
@@ -3425,7 +3425,7 @@
         <v>337</v>
       </c>
       <c r="C34">
-        <v>685</v>
+        <v>426</v>
       </c>
       <c r="D34" t="s">
         <v>270</v>
@@ -3442,7 +3442,7 @@
         <v>339</v>
       </c>
       <c r="C35">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="D35" t="s">
         <v>273</v>
@@ -3459,7 +3459,7 @@
         <v>341</v>
       </c>
       <c r="C36">
-        <v>739</v>
+        <v>103</v>
       </c>
       <c r="D36" t="s">
         <v>276</v>
@@ -3476,7 +3476,7 @@
         <v>343</v>
       </c>
       <c r="C37">
-        <v>379</v>
+        <v>489</v>
       </c>
       <c r="D37" t="s">
         <v>279</v>
@@ -3493,7 +3493,7 @@
         <v>345</v>
       </c>
       <c r="C38">
-        <v>380</v>
+        <v>242</v>
       </c>
       <c r="D38" t="s">
         <v>270</v>
@@ -3510,7 +3510,7 @@
         <v>347</v>
       </c>
       <c r="C39">
-        <v>472</v>
+        <v>131</v>
       </c>
       <c r="D39" t="s">
         <v>273</v>
@@ -3527,7 +3527,7 @@
         <v>349</v>
       </c>
       <c r="C40">
-        <v>213</v>
+        <v>47</v>
       </c>
       <c r="D40" t="s">
         <v>276</v>
@@ -3544,7 +3544,7 @@
         <v>351</v>
       </c>
       <c r="C41">
-        <v>612</v>
+        <v>457</v>
       </c>
       <c r="D41" t="s">
         <v>279</v>
@@ -3561,7 +3561,7 @@
         <v>353</v>
       </c>
       <c r="C42">
-        <v>471</v>
+        <v>100</v>
       </c>
       <c r="D42" t="s">
         <v>270</v>
@@ -3578,7 +3578,7 @@
         <v>355</v>
       </c>
       <c r="C43">
-        <v>624</v>
+        <v>159</v>
       </c>
       <c r="D43" t="s">
         <v>273</v>
@@ -3595,7 +3595,7 @@
         <v>357</v>
       </c>
       <c r="C44">
-        <v>882</v>
+        <v>168</v>
       </c>
       <c r="D44" t="s">
         <v>276</v>
@@ -3612,7 +3612,7 @@
         <v>359</v>
       </c>
       <c r="C45">
-        <v>137</v>
+        <v>76</v>
       </c>
       <c r="D45" t="s">
         <v>279</v>
@@ -3629,7 +3629,7 @@
         <v>361</v>
       </c>
       <c r="C46">
-        <v>449</v>
+        <v>911</v>
       </c>
       <c r="D46" t="s">
         <v>270</v>
@@ -3646,7 +3646,7 @@
         <v>363</v>
       </c>
       <c r="C47">
-        <v>136</v>
+        <v>538</v>
       </c>
       <c r="D47" t="s">
         <v>273</v>
@@ -3663,7 +3663,7 @@
         <v>365</v>
       </c>
       <c r="C48">
-        <v>654</v>
+        <v>242</v>
       </c>
       <c r="D48" t="s">
         <v>276</v>
@@ -3680,7 +3680,7 @@
         <v>367</v>
       </c>
       <c r="C49">
-        <v>642</v>
+        <v>244</v>
       </c>
       <c r="D49" t="s">
         <v>279</v>
@@ -3697,7 +3697,7 @@
         <v>369</v>
       </c>
       <c r="C50">
-        <v>475</v>
+        <v>723</v>
       </c>
       <c r="D50" t="s">
         <v>270</v>
@@ -3714,7 +3714,7 @@
         <v>371</v>
       </c>
       <c r="C51">
-        <v>621</v>
+        <v>870</v>
       </c>
       <c r="D51" t="s">
         <v>273</v>

</xml_diff>